<commit_message>
Remove breeding_migration col from data for now.
</commit_message>
<xml_diff>
--- a/R/auxiliary_scripts/aux_schema_cols.xlsx
+++ b/R/auxiliary_scripts/aux_schema_cols.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://michiganstate-my.sharepoint.com/personal/kapsarke_msu_edu/Documents/Research/AvianMetaNetwork/AvianMetaNetwork/R/auxiliary_scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{A7E1EE30-6DA6-4551-A03C-270667897E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D514788-98C3-42A1-90B5-572987CBA310}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{A7E1EE30-6DA6-4551-A03C-270667897E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0526B8DE-001C-46BE-A0C8-DC48A0A670DB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1F04E687-57B4-4B53-968B-A3F09457A236}"/>
+    <workbookView xWindow="28680" yWindow="300" windowWidth="25440" windowHeight="15270" xr2:uid="{1F04E687-57B4-4B53-968B-A3F09457A236}"/>
   </bookViews>
   <sheets>
     <sheet name="aux_schema_cols" sheetId="1" r:id="rId1"/>
@@ -821,6 +821,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1142,7 +1146,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="10" width="12.7109375" customWidth="1"/>
+    <col min="2" max="9" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -2419,7 +2424,7 @@
         <v>1</v>
       </c>
       <c r="K36">
-        <f t="shared" ref="K36:K67" si="1">COUNTIF(B36:J36, TRUE)</f>
+        <f t="shared" ref="K36:K60" si="1">COUNTIF(B36:J36, TRUE)</f>
         <v>2</v>
       </c>
     </row>
@@ -3303,6 +3308,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>